<commit_message>
isotopos ok, empezando dbhd
</commit_message>
<xml_diff>
--- a/Sumaco/Sumaco_cellulose.xlsx
+++ b/Sumaco/Sumaco_cellulose.xlsx
@@ -486,7 +486,7 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>PlotID</t>
+          <t>Type</t>
         </is>
       </c>
     </row>
@@ -535,7 +535,7 @@
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>SUM_09</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -586,7 +586,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>SUM_01</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>SUM_09</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -682,7 +682,7 @@
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
-          <t>SUM_9.0</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -733,7 +733,7 @@
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr">
         <is>
-          <t>SUM_09</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -784,7 +784,7 @@
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr">
         <is>
-          <t>SUM_10</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -833,7 +833,7 @@
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr">
         <is>
-          <t>SUM_10</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -886,7 +886,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>SUM_10</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -935,7 +935,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>SUM_10.0</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -984,7 +984,7 @@
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr">
         <is>
-          <t>SUM_10</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -1037,7 +1037,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>SUM_10</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -1092,7 +1092,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>SUM_10</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -1143,7 +1143,7 @@
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr">
         <is>
-          <t>SUM_10</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -1184,7 +1184,7 @@
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr">
         <is>
-          <t>SUM_nan</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -1233,7 +1233,7 @@
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr">
         <is>
-          <t>SUM_10</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -1284,7 +1284,7 @@
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr">
         <is>
-          <t>SUM_11</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -1337,7 +1337,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>SUM_11</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -1390,7 +1390,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>SUM_11</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -1441,7 +1441,7 @@
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr">
         <is>
-          <t>SUM_11</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -1490,7 +1490,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>SUM_11</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -1541,7 +1541,7 @@
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr">
         <is>
-          <t>SUM_11</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -1592,7 +1592,7 @@
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr">
         <is>
-          <t>SUM_11</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -1641,7 +1641,7 @@
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr">
         <is>
-          <t>SUM_11</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -1692,7 +1692,7 @@
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr">
         <is>
-          <t>SUM_11</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -1743,7 +1743,7 @@
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr">
         <is>
-          <t>SUM_11</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -1794,7 +1794,7 @@
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr">
         <is>
-          <t>SUM_12</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>SUM_12</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -1896,7 +1896,7 @@
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr">
         <is>
-          <t>SUM_12</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -1951,7 +1951,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>SUM_12</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -2000,7 +2000,7 @@
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr">
         <is>
-          <t>SUM_12</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -2051,7 +2051,7 @@
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr">
         <is>
-          <t>SUM_12</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -2104,7 +2104,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>SUM_12</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -2149,7 +2149,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>SUM_nan</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -2200,7 +2200,7 @@
       <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr">
         <is>
-          <t>SUM_12</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -2251,7 +2251,7 @@
       <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr">
         <is>
-          <t>SUM_12</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -2304,7 +2304,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>SUM_13</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -2353,7 +2353,7 @@
       <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr">
         <is>
-          <t>SUM_13</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -2402,7 +2402,7 @@
       <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr">
         <is>
-          <t>SUM_13</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -2447,7 +2447,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>SUM_nan</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -2500,7 +2500,7 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>SUM_13</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -2549,7 +2549,7 @@
       <c r="L42" t="inlineStr"/>
       <c r="M42" t="inlineStr">
         <is>
-          <t>SUM_13.0</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -2598,7 +2598,7 @@
       <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr">
         <is>
-          <t>SUM_13</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -2647,7 +2647,7 @@
       <c r="L44" t="inlineStr"/>
       <c r="M44" t="inlineStr">
         <is>
-          <t>SUM_13</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -2696,7 +2696,7 @@
       <c r="L45" t="inlineStr"/>
       <c r="M45" t="inlineStr">
         <is>
-          <t>SUM_13</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -2745,7 +2745,7 @@
       <c r="L46" t="inlineStr"/>
       <c r="M46" t="inlineStr">
         <is>
-          <t>SUM_13</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -2796,7 +2796,7 @@
       <c r="L47" t="inlineStr"/>
       <c r="M47" t="inlineStr">
         <is>
-          <t>SUM_p09</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -2847,7 +2847,7 @@
       <c r="L48" t="inlineStr"/>
       <c r="M48" t="inlineStr">
         <is>
-          <t>SUM_p09</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -2896,7 +2896,7 @@
       <c r="L49" t="inlineStr"/>
       <c r="M49" t="inlineStr">
         <is>
-          <t>SUM_p09</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -2949,7 +2949,7 @@
       <c r="L50" t="inlineStr"/>
       <c r="M50" t="inlineStr">
         <is>
-          <t>SUM_p09</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -3002,7 +3002,7 @@
       <c r="L51" t="inlineStr"/>
       <c r="M51" t="inlineStr">
         <is>
-          <t>SUM_p09</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -3055,7 +3055,7 @@
       <c r="L52" t="inlineStr"/>
       <c r="M52" t="inlineStr">
         <is>
-          <t>SUM_p09</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -3108,7 +3108,7 @@
       <c r="L53" t="inlineStr"/>
       <c r="M53" t="inlineStr">
         <is>
-          <t>SUM_p09</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -3159,7 +3159,7 @@
       <c r="L54" t="inlineStr"/>
       <c r="M54" t="inlineStr">
         <is>
-          <t>SUM_p10</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       <c r="L55" t="inlineStr"/>
       <c r="M55" t="inlineStr">
         <is>
-          <t>SUM_p10</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -3261,7 +3261,7 @@
       <c r="L56" t="inlineStr"/>
       <c r="M56" t="inlineStr">
         <is>
-          <t>SUM_p10</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -3312,7 +3312,7 @@
       <c r="L57" t="inlineStr"/>
       <c r="M57" t="inlineStr">
         <is>
-          <t>SUM_p10</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -3363,7 +3363,7 @@
       <c r="L58" t="inlineStr"/>
       <c r="M58" t="inlineStr">
         <is>
-          <t>SUM_p10</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -3414,7 +3414,7 @@
       <c r="L59" t="inlineStr"/>
       <c r="M59" t="inlineStr">
         <is>
-          <t>SUM_p10</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -3465,7 +3465,7 @@
       <c r="L60" t="inlineStr"/>
       <c r="M60" t="inlineStr">
         <is>
-          <t>SUM_p10</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -3516,7 +3516,7 @@
       <c r="L61" t="inlineStr"/>
       <c r="M61" t="inlineStr">
         <is>
-          <t>SUM_10.0</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -3569,7 +3569,7 @@
       <c r="L62" t="inlineStr"/>
       <c r="M62" t="inlineStr">
         <is>
-          <t>SUM_p10</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -3620,7 +3620,7 @@
       <c r="L63" t="inlineStr"/>
       <c r="M63" t="inlineStr">
         <is>
-          <t>SUM_p11</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -3671,7 +3671,7 @@
       <c r="L64" t="inlineStr"/>
       <c r="M64" t="inlineStr">
         <is>
-          <t>SUM_p11</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -3722,7 +3722,7 @@
       <c r="L65" t="inlineStr"/>
       <c r="M65" t="inlineStr">
         <is>
-          <t>SUM_p11</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -3773,7 +3773,7 @@
       <c r="L66" t="inlineStr"/>
       <c r="M66" t="inlineStr">
         <is>
-          <t>SUM_p11</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -3820,7 +3820,7 @@
       <c r="L67" t="inlineStr"/>
       <c r="M67" t="inlineStr">
         <is>
-          <t>SUM_p11</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -3871,7 +3871,7 @@
       <c r="L68" t="inlineStr"/>
       <c r="M68" t="inlineStr">
         <is>
-          <t>SUM_p11</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -3922,7 +3922,7 @@
       <c r="L69" t="inlineStr"/>
       <c r="M69" t="inlineStr">
         <is>
-          <t>SUM_p11</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -3973,7 +3973,7 @@
       <c r="L70" t="inlineStr"/>
       <c r="M70" t="inlineStr">
         <is>
-          <t>SUM_p11</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -4018,7 +4018,7 @@
       <c r="L71" t="inlineStr"/>
       <c r="M71" t="inlineStr">
         <is>
-          <t>SUM_p11</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -4069,7 +4069,7 @@
       <c r="L72" t="inlineStr"/>
       <c r="M72" t="inlineStr">
         <is>
-          <t>SUM_p12</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -4120,7 +4120,7 @@
       <c r="L73" t="inlineStr"/>
       <c r="M73" t="inlineStr">
         <is>
-          <t>SUM_p12</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -4171,7 +4171,7 @@
       <c r="L74" t="inlineStr"/>
       <c r="M74" t="inlineStr">
         <is>
-          <t>SUM_p12</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -4222,7 +4222,7 @@
       <c r="L75" t="inlineStr"/>
       <c r="M75" t="inlineStr">
         <is>
-          <t>SUM_p12</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -4273,7 +4273,7 @@
       <c r="L76" t="inlineStr"/>
       <c r="M76" t="inlineStr">
         <is>
-          <t>SUM_p12</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -4326,7 +4326,7 @@
       <c r="L77" t="inlineStr"/>
       <c r="M77" t="inlineStr">
         <is>
-          <t>SUM_p12</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       <c r="L78" t="inlineStr"/>
       <c r="M78" t="inlineStr">
         <is>
-          <t>SUM_p12</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -4426,7 +4426,7 @@
       <c r="L79" t="inlineStr"/>
       <c r="M79" t="inlineStr">
         <is>
-          <t>SUM_p12</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -4473,7 +4473,7 @@
       <c r="L80" t="inlineStr"/>
       <c r="M80" t="inlineStr">
         <is>
-          <t>SUM_p16</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -4520,7 +4520,7 @@
       <c r="L81" t="inlineStr"/>
       <c r="M81" t="inlineStr">
         <is>
-          <t>SUM_p16</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -4571,7 +4571,7 @@
       <c r="L82" t="inlineStr"/>
       <c r="M82" t="inlineStr">
         <is>
-          <t>SUM_p16</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -4618,7 +4618,7 @@
       <c r="L83" t="inlineStr"/>
       <c r="M83" t="inlineStr">
         <is>
-          <t>SUM_p16</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -4665,7 +4665,7 @@
       <c r="L84" t="inlineStr"/>
       <c r="M84" t="inlineStr">
         <is>
-          <t>SUM_p16</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -4712,7 +4712,7 @@
       <c r="L85" t="inlineStr"/>
       <c r="M85" t="inlineStr">
         <is>
-          <t>SUM_p16</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -4759,7 +4759,7 @@
       <c r="L86" t="inlineStr"/>
       <c r="M86" t="inlineStr">
         <is>
-          <t>SUM_p18</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -4806,7 +4806,7 @@
       <c r="L87" t="inlineStr"/>
       <c r="M87" t="inlineStr">
         <is>
-          <t>SUM_p18</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -4853,7 +4853,7 @@
       <c r="L88" t="inlineStr"/>
       <c r="M88" t="inlineStr">
         <is>
-          <t>SUM_p18</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -4896,7 +4896,7 @@
       <c r="L89" t="inlineStr"/>
       <c r="M89" t="inlineStr">
         <is>
-          <t>SUM_p18</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -4949,7 +4949,7 @@
       <c r="L90" t="inlineStr"/>
       <c r="M90" t="inlineStr">
         <is>
-          <t>SUM_p18</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -4994,7 +4994,7 @@
       <c r="L91" t="inlineStr"/>
       <c r="M91" t="inlineStr">
         <is>
-          <t>SUM_p18</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>
@@ -5007,7 +5007,11 @@
           <t>p12-3686</t>
         </is>
       </c>
-      <c r="C92" t="inlineStr"/>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Moracea</t>
+        </is>
+      </c>
       <c r="D92" t="inlineStr"/>
       <c r="E92" t="inlineStr"/>
       <c r="F92" t="n">
@@ -5019,7 +5023,9 @@
       <c r="H92" t="n">
         <v>12</v>
       </c>
-      <c r="I92" t="inlineStr"/>
+      <c r="I92" t="n">
+        <v>2025</v>
+      </c>
       <c r="J92" t="inlineStr"/>
       <c r="K92" t="n">
         <v>3686</v>
@@ -5027,7 +5033,7 @@
       <c r="L92" t="inlineStr"/>
       <c r="M92" t="inlineStr">
         <is>
-          <t>SUM_12.0</t>
+          <t>leaf pulverized</t>
         </is>
       </c>
     </row>

</xml_diff>